<commit_message>
Corregir Excel de importación, actualizar manuales y agregar enlace del video
</commit_message>
<xml_diff>
--- a/Proyecto/Fase2/techcore-odoo/1_Productos_Odoo.xlsx
+++ b/Proyecto/Fase2/techcore-odoo/1_Productos_Odoo.xlsx
@@ -417,56 +417,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>default_code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>categ_id</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>list_price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>standard_price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>detailed_type</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>sale_ok</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>purchase_ok</t>
         </is>
@@ -475,680 +481,780 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>techcore_prod_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>PROD-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Intel Core i9-13900K</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Procesador</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>All / Procesador</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>650</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>500</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>techcore_prod_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>PROD-002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>AMD Ryzen 9 7950X</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Procesador</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>All / Procesador</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>600</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>480</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>techcore_prod_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>PROD-003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Corsair Vengeance 32GB DDR5</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Memoria RAM</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>All / Memoria RAM</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>150</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>100</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>techcore_prod_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>PROD-004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Kingston Fury Beast 16GB DDR4</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Memoria RAM</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>All / Memoria RAM</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
         <v>60</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>40</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>techcore_prod_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>PROD-005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Samsung 990 PRO 2TB NVMe</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SSD</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>All / SSD</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>200</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>140</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>techcore_prod_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>PROD-006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>WD Black SN850X 1TB NVMe</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SSD</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>All / SSD</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
         <v>120</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>80</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>techcore_prod_007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>PROD-007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Cisco Catalyst 2960-X 24 Port</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Switch</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>All / Switch</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
         <v>800</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>600</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>techcore_prod_008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>PROD-008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Ubiquiti UniFi Switch 48 PoE</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Switch</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>All / Switch</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
         <v>1100</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>850</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>1</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>techcore_prod_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>PROD-009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Dell PowerEdge R750</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Servidor</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>All / Servidor</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
         <v>4500</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>3500</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>1</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>techcore_prod_010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>PROD-010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>HPE ProLiant DL380 Gen10</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Servidor</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>All / Servidor</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
         <v>4200</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>3200</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>1</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>techcore_prod_011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>PROD-011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>ASUS ROG Maximus Z790 Hero</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Tarjeta Madre</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>All / Tarjeta Madre</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
         <v>600</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>450</v>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>1</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>techcore_prod_012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>PROD-012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>MSI MAG B650 Tomahawk WiFi</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Tarjeta Madre</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>All / Tarjeta Madre</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
         <v>250</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>180</v>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>1</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>techcore_prod_013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>PROD-013</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Intel Core i5-13600K</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Procesador</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>All / Procesador</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
         <v>320</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>250</v>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>1</v>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>techcore_prod_014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>PROD-014</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>AMD Ryzen 5 7600X</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Procesador</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>All / Procesador</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
         <v>280</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>220</v>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>1</v>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>techcore_prod_015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>PROD-015</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>G.Skill Trident Z5 RGB 64GB</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Memoria RAM</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>All / Memoria RAM</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
         <v>280</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>200</v>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>1</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>techcore_prod_016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>PROD-016</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Crucial P3 Plus 4TB NVMe</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>SSD</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>All / SSD</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
         <v>250</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>190</v>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>1</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>techcore_prod_017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>PROD-017</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>TP-Link TL-SG108E 8 Port</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Switch</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>All / Switch</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
         <v>40</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>25</v>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>1</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>techcore_prod_018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>PROD-018</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Lenovo ThinkSystem SR650</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Servidor</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>All / Servidor</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
         <v>3800</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>2900</v>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>1</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>techcore_prod_019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>PROD-019</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Gigabyte X670E AORUS Master</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Tarjeta Madre</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>All / Tarjeta Madre</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
         <v>500</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>380</v>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>1</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>techcore_prod_020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>PROD-020</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Seagate IronWolf Pro 18TB</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Disco Duro</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>All / Disco Duro</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
         <v>350</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>260</v>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>1</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
       </c>
       <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>